<commit_message>
Proof of concept of merging in existing metadata from the provided spreadsheet
</commit_message>
<xml_diff>
--- a/examples/output.xlsx
+++ b/examples/output.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="4"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="turn" sheetId="1" state="visible" r:id="rId3"/>
@@ -189,8 +189,12 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -390,231 +394,231 @@
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="0" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="0" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="0" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="0" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="C2" s="0" t="n">
+      <c r="A2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" s="1" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="C3" s="0" t="n">
-        <v>2</v>
-      </c>
-      <c r="D3" s="0" t="s">
+      <c r="A3" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="D3" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="E3" s="0" t="s">
+      <c r="E3" s="1" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="C4" s="0" t="n">
+      <c r="A4" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C4" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="D4" s="0" t="s">
+      <c r="D4" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="E4" s="0" t="s">
+      <c r="E4" s="1" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="C5" s="0" t="n">
+      <c r="A5" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C5" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="D5" s="0" t="s">
+      <c r="D5" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="E5" s="0" t="s">
+      <c r="E5" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
-        <v>5</v>
-      </c>
-      <c r="B6" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="C6" s="0" t="n">
-        <v>5</v>
-      </c>
-      <c r="D6" s="0" t="s">
+      <c r="A6" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C6" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="D6" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="E6" s="0" t="s">
+      <c r="E6" s="1" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
-        <v>5</v>
-      </c>
-      <c r="B7" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="C7" s="0" t="n">
+      <c r="A7" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B7" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="D7" s="0" t="s">
+      <c r="D7" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="E7" s="0" t="s">
+      <c r="E7" s="1" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="s">
-        <v>5</v>
-      </c>
-      <c r="B8" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="C8" s="0" t="n">
+      <c r="A8" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B8" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C8" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="D8" s="0" t="s">
+      <c r="D8" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="E8" s="0" t="s">
+      <c r="E8" s="1" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="s">
-        <v>5</v>
-      </c>
-      <c r="B9" s="0" t="n">
-        <v>2</v>
-      </c>
-      <c r="C9" s="0" t="n">
+      <c r="A9" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B9" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="C9" s="1" t="n">
         <v>9</v>
       </c>
-      <c r="D9" s="0" t="s">
+      <c r="D9" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="E9" s="0" t="s">
+      <c r="E9" s="1" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="s">
-        <v>5</v>
-      </c>
-      <c r="B10" s="0" t="n">
-        <v>2</v>
-      </c>
-      <c r="C10" s="0" t="n">
+      <c r="A10" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B10" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="C10" s="1" t="n">
         <v>10</v>
       </c>
-      <c r="D10" s="0" t="s">
+      <c r="D10" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="E10" s="0" t="s">
+      <c r="E10" s="1" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="s">
-        <v>5</v>
-      </c>
-      <c r="B11" s="0" t="n">
-        <v>2</v>
-      </c>
-      <c r="C11" s="0" t="n">
+      <c r="A11" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B11" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="C11" s="1" t="n">
         <v>11</v>
       </c>
-      <c r="D11" s="0" t="s">
+      <c r="D11" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="E11" s="0" t="s">
+      <c r="E11" s="1" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="0" t="s">
-        <v>5</v>
-      </c>
-      <c r="B12" s="0" t="n">
-        <v>2</v>
-      </c>
-      <c r="C12" s="0" t="n">
+      <c r="A12" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B12" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="C12" s="1" t="n">
         <v>12</v>
       </c>
-      <c r="D12" s="0" t="s">
+      <c r="D12" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="E12" s="0" t="s">
+      <c r="E12" s="1" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="0" t="s">
-        <v>5</v>
-      </c>
-      <c r="B13" s="0" t="n">
-        <v>2</v>
-      </c>
-      <c r="C13" s="0" t="n">
+      <c r="A13" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B13" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="C13" s="1" t="n">
         <v>13</v>
       </c>
-      <c r="D13" s="0" t="s">
+      <c r="D13" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="E13" s="0" t="s">
+      <c r="E13" s="1" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="0" t="s">
-        <v>5</v>
-      </c>
-      <c r="B14" s="0" t="n">
-        <v>2</v>
-      </c>
-      <c r="C14" s="0" t="n">
+      <c r="A14" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B14" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="C14" s="1" t="n">
         <v>14</v>
       </c>
-      <c r="E14" s="0" t="s">
+      <c r="E14" s="1" t="s">
         <v>20</v>
       </c>
     </row>
@@ -638,66 +642,66 @@
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" s="1" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
-        <v>5</v>
-      </c>
-      <c r="C2" s="0" t="n">
+      <c r="A2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="1" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3" s="0" t="s">
+      <c r="A3" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="0" t="n">
-        <v>5</v>
-      </c>
-      <c r="D3" s="0" t="n">
+      <c r="C3" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="D3" s="1" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4" s="0" t="s">
+      <c r="A4" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C4" s="0" t="n">
+      <c r="C4" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="D4" s="0" t="n">
+      <c r="D4" s="1" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5" s="0" t="s">
+      <c r="A5" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C5" s="0" t="n">
+      <c r="C5" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="D5" s="0" t="n">
+      <c r="D5" s="1" t="n">
         <v>3</v>
       </c>
     </row>
@@ -721,44 +725,44 @@
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="0" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="0" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" s="1" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="C2" s="0" t="n">
+      <c r="A2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="D2" s="0" t="s">
+      <c r="D2" s="1" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3" s="0" t="n">
-        <v>2</v>
-      </c>
-      <c r="C3" s="0" t="n">
+      <c r="A3" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="D3" s="0" t="s">
+      <c r="D3" s="1" t="s">
         <v>25</v>
       </c>
     </row>
@@ -782,18 +786,18 @@
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" s="0" t="n">
+      <c r="A2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="1" t="n">
         <v>13</v>
       </c>
     </row>
@@ -816,35 +820,35 @@
   <dimension ref="A1:B4"/>
   <sheetFormatPr defaultColWidth="10.16015625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
-    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" s="0" t="s">
+    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" s="0" t="s">
+    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="n">
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="1" t="s">
         <v>29</v>
       </c>
     </row>

</xml_diff>